<commit_message>
added student data as a excel file
</commit_message>
<xml_diff>
--- a/student_data.xlsx
+++ b/student_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnudipCOA\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnudipCOA\project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A31EF01-85F2-48AA-A14D-695FED19577D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85284044-6129-4CBC-B3B9-0D3EBEBE9F93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4620" yWindow="3510" windowWidth="18000" windowHeight="9270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
     <t>HTML</t>
   </si>
   <si>
-    <t>SQL</t>
+    <t>java</t>
   </si>
 </sst>
 </file>

</xml_diff>